<commit_message>
Fix product links: use only verified URLs, leave prices empty
Replaces constructed (404-prone) product URLs with search-index-verified
links. Adds column R for distributor shop pages (price source) alongside
column Q (manufacturer page). Price column G left empty for the added
positions so it can be filled directly from the linked pages.

https://claude.ai/code/session_01K5i3UW8gwbQYbMAvbFAQPj
</commit_message>
<xml_diff>
--- a/Kostenschaetzung.xlsx
+++ b/Kostenschaetzung.xlsx
@@ -19,7 +19,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0.00 €"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,13 +48,17 @@
       <sz val="10"/>
     </font>
     <font>
+      <color rgb="000563C1"/>
+      <sz val="9"/>
+      <u val="single"/>
+    </font>
+    <font>
       <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
@@ -91,7 +95,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
@@ -120,26 +124,34 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -484,16 +496,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C4:AA66"/>
+  <dimension ref="C4:AA68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="35" customWidth="1" min="16" max="16"/>
-    <col width="50" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="46" customWidth="1" min="17" max="17"/>
+    <col width="46" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="4">
@@ -522,21 +535,31 @@
           <t>GP [€]</t>
         </is>
       </c>
+      <c r="P4" s="12" t="inlineStr">
+        <is>
+          <t>Datenblatt</t>
+        </is>
+      </c>
       <c r="Q4" s="12" t="inlineStr">
         <is>
-          <t>Produkt-Link</t>
+          <t>Hersteller-Link</t>
+        </is>
+      </c>
+      <c r="R4" s="12" t="inlineStr">
+        <is>
+          <t>Händler-Link (Preisquelle)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="210" customHeight="1">
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">UP, Daten-Anschlussdose, Cat.6, 2x RJ45, WLAN Öffentlich 
 </t>
         </is>
       </c>
       <c r="D5" s="2" t="n"/>
-      <c r="E5" s="20" t="n">
+      <c r="E5" s="14" t="n">
         <v>102</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -544,7 +567,7 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G5" s="13" t="n">
+      <c r="G5" s="15" t="n">
         <v>37.31</v>
       </c>
       <c r="H5" s="2" t="n"/>
@@ -554,7 +577,7 @@
       <c r="L5" s="2" t="n"/>
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="n"/>
-      <c r="O5" s="13">
+      <c r="O5" s="15">
         <f>E5*G5</f>
         <v/>
       </c>
@@ -563,36 +586,40 @@
           <t>https://ibgoetz.sharepoint.com/:b:/s/IBG_Gewerbe/IQC30NCBU9A_TKQDbCNJgepgAZR8CeUhfyKy5Hk9NjtHBN0?e=96lFEy</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr">
+      <c r="Q5" s="16" t="inlineStr">
         <is>
           <t>https://www.metz-connect.com/home/produkte/p-cabling/anschlussdosen/rj45.ea.de.html</t>
         </is>
       </c>
-      <c r="R5" s="2" t="n"/>
+      <c r="R5" s="16" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Datennetzwerktechnik/Netzwerkkomponente/Kommunikationsanschlussdosen/Kupfer/Metz-Connect-Anschlussdose-Cat-6A-TN-E-DATmod-2Up0::144962.html</t>
+        </is>
+      </c>
       <c r="S5" s="2" t="n"/>
       <c r="T5" s="2" t="n"/>
       <c r="U5" s="2" t="n"/>
       <c r="V5" s="2" t="n"/>
       <c r="W5" s="2" t="n"/>
-      <c r="Y5" s="14" t="inlineStr">
+      <c r="Y5" s="17" t="inlineStr">
         <is>
           <t>datendosen abzahl gesamt:</t>
         </is>
       </c>
-      <c r="Z5" s="14" t="n"/>
+      <c r="Z5" s="17" t="n"/>
       <c r="AA5" t="n">
         <v>982</v>
       </c>
     </row>
     <row r="6" ht="210" customHeight="1">
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">UP, Daten-Anschlussdose, Cat.6, 2x RJ45, Drucker 
 </t>
         </is>
       </c>
       <c r="D6" s="2" t="n"/>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="14" t="n">
         <v>2</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -600,7 +627,7 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G6" s="13" t="n">
+      <c r="G6" s="15" t="n">
         <v>37.31</v>
       </c>
       <c r="H6" s="2" t="n"/>
@@ -610,7 +637,7 @@
       <c r="L6" s="2" t="n"/>
       <c r="M6" s="2" t="n"/>
       <c r="N6" s="2" t="n"/>
-      <c r="O6" s="13">
+      <c r="O6" s="15">
         <f>E6*G6</f>
         <v/>
       </c>
@@ -619,29 +646,33 @@
           <t>https://ibgoetz.sharepoint.com/:b:/s/IBG_Gewerbe/IQC30NCBU9A_TKQDbCNJgepgAZR8CeUhfyKy5Hk9NjtHBN0?e=96lFEy</t>
         </is>
       </c>
-      <c r="Q6" s="2" t="inlineStr">
+      <c r="Q6" s="16" t="inlineStr">
         <is>
           <t>https://www.metz-connect.com/home/produkte/p-cabling/anschlussdosen/rj45.ea.de.html</t>
         </is>
       </c>
-      <c r="R6" s="2" t="n"/>
+      <c r="R6" s="16" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Datennetzwerktechnik/Netzwerkkomponente/Kommunikationsanschlussdosen/Kupfer/Metz-Connect-Anschlussdose-Cat-6A-TN-E-DATmod-2Up0::144962.html</t>
+        </is>
+      </c>
       <c r="S6" s="2" t="n"/>
       <c r="T6" s="2" t="n"/>
       <c r="U6" s="2" t="n"/>
       <c r="V6" s="2" t="n"/>
       <c r="W6" s="2" t="n"/>
-      <c r="Y6" s="14" t="n"/>
-      <c r="Z6" s="14" t="n"/>
+      <c r="Y6" s="17" t="n"/>
+      <c r="Z6" s="17" t="n"/>
     </row>
     <row r="7" ht="210" customHeight="1">
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">UP, Daten-Anschlussdose, Cat.6, 2x RJ45, Technik 
 </t>
         </is>
       </c>
       <c r="D7" s="2" t="n"/>
-      <c r="E7" s="20" t="n">
+      <c r="E7" s="14" t="n">
         <v>14</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -649,7 +680,7 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G7" s="13" t="n">
+      <c r="G7" s="15" t="n">
         <v>37.31</v>
       </c>
       <c r="H7" s="2" t="n"/>
@@ -659,7 +690,7 @@
       <c r="L7" s="2" t="n"/>
       <c r="M7" s="2" t="n"/>
       <c r="N7" s="2" t="n"/>
-      <c r="O7" s="13">
+      <c r="O7" s="15">
         <f>E7*G7</f>
         <v/>
       </c>
@@ -668,29 +699,33 @@
           <t>https://ibgoetz.sharepoint.com/:b:/s/IBG_Gewerbe/IQC30NCBU9A_TKQDbCNJgepgAZR8CeUhfyKy5Hk9NjtHBN0?e=96lFEy</t>
         </is>
       </c>
-      <c r="Q7" s="2" t="inlineStr">
+      <c r="Q7" s="16" t="inlineStr">
         <is>
           <t>https://www.metz-connect.com/home/produkte/p-cabling/anschlussdosen/rj45.ea.de.html</t>
         </is>
       </c>
-      <c r="R7" s="2" t="n"/>
+      <c r="R7" s="16" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Datennetzwerktechnik/Netzwerkkomponente/Kommunikationsanschlussdosen/Kupfer/Metz-Connect-Anschlussdose-Cat-6A-TN-E-DATmod-2Up0::144962.html</t>
+        </is>
+      </c>
       <c r="S7" s="2" t="n"/>
       <c r="T7" s="2" t="n"/>
       <c r="U7" s="2" t="n"/>
       <c r="V7" s="2" t="n"/>
       <c r="W7" s="2" t="n"/>
-      <c r="Y7" s="14" t="n"/>
-      <c r="Z7" s="14" t="n"/>
+      <c r="Y7" s="17" t="n"/>
+      <c r="Z7" s="17" t="n"/>
     </row>
     <row r="8" ht="210" customHeight="1">
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">AP, Daten-Anschlussdose, Cat.6, 2x RJ45, MÜK 
 </t>
         </is>
       </c>
       <c r="D8" s="2" t="n"/>
-      <c r="E8" s="20" t="n">
+      <c r="E8" s="14" t="n">
         <v>57</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -698,7 +733,7 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G8" s="13" t="n">
+      <c r="G8" s="15" t="n">
         <v>37.31</v>
       </c>
       <c r="H8" s="2" t="n"/>
@@ -708,7 +743,7 @@
       <c r="L8" s="2" t="n"/>
       <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="n"/>
-      <c r="O8" s="13">
+      <c r="O8" s="15">
         <f>E8*G8</f>
         <v/>
       </c>
@@ -717,21 +752,25 @@
           <t>https://ibgoetz.sharepoint.com/:b:/s/IBG_Gewerbe/IQC30NCBU9A_TKQDbCNJgepgAZR8CeUhfyKy5Hk9NjtHBN0?e=96lFEy</t>
         </is>
       </c>
-      <c r="Q8" s="2" t="inlineStr">
+      <c r="Q8" s="16" t="inlineStr">
         <is>
           <t>https://www.metz-connect.com/home/produkte/p-cabling/anschlussdosen/rj45.ea.de.html</t>
         </is>
       </c>
-      <c r="R8" s="2" t="n"/>
+      <c r="R8" s="16" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Datennetzwerktechnik/Netzwerkkomponente/Kommunikationsanschlussdosen/Kupfer/Metz-Connect-Anschlussdose-Cat-6A-TN-E-DATmod-2Up0::144962.html</t>
+        </is>
+      </c>
       <c r="S8" s="2" t="n"/>
       <c r="T8" s="2" t="n"/>
       <c r="U8" s="2" t="n"/>
       <c r="V8" s="2" t="n"/>
       <c r="W8" s="2" t="n"/>
-      <c r="Y8" s="14" t="n"/>
+      <c r="Y8" s="17" t="n"/>
     </row>
     <row r="9" ht="210" customHeight="1">
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Daten-Anschlussdose Cat.6 2x RJ45</t>
         </is>
@@ -744,10 +783,10 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G9" s="13" t="n">
+      <c r="G9" s="15" t="n">
         <v>37.31</v>
       </c>
-      <c r="O9" s="13">
+      <c r="O9" s="15">
         <f>E9*G9</f>
         <v/>
       </c>
@@ -756,19 +795,24 @@
           <t>https://ibgoetz.sharepoint.com/:b:/s/IBG_Gewerbe/IQC30NCBU9A_TKQDbCNJgepgAZR8CeUhfyKy5Hk9NjtHBN0?e=96lFEy</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="Q9" s="19" t="inlineStr">
         <is>
           <t>https://www.metz-connect.com/home/produkte/p-cabling/anschlussdosen/rj45.ea.de.html</t>
         </is>
       </c>
+      <c r="R9" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Datennetzwerktechnik/Netzwerkkomponente/Kommunikationsanschlussdosen/Kupfer/Metz-Connect-Anschlussdose-Cat-6A-TN-E-DATmod-2Up0::144962.html</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="210" customHeight="1">
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">UP, Daten-Anschlussdose, Cat.6, 2x RJ45, Kasse </t>
         </is>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="14" t="n">
         <v>5</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -776,10 +820,10 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G10" s="13" t="n">
+      <c r="G10" s="15" t="n">
         <v>37.31</v>
       </c>
-      <c r="O10" s="13">
+      <c r="O10" s="15">
         <f>E10*G10</f>
         <v/>
       </c>
@@ -788,19 +832,24 @@
           <t>https://ibgoetz.sharepoint.com/:b:/s/IBG_Gewerbe/IQC30NCBU9A_TKQDbCNJgepgAZR8CeUhfyKy5Hk9NjtHBN0?e=96lFEy</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="Q10" s="19" t="inlineStr">
         <is>
           <t>https://www.metz-connect.com/home/produkte/p-cabling/anschlussdosen/rj45.ea.de.html</t>
         </is>
       </c>
+      <c r="R10" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Datennetzwerktechnik/Netzwerkkomponente/Kommunikationsanschlussdosen/Kupfer/Metz-Connect-Anschlussdose-Cat-6A-TN-E-DATmod-2Up0::144962.html</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="210" customHeight="1">
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">UP, Daten-Anschlussdose, Cat.6, 2x RJ45, WLAN Mieter </t>
         </is>
       </c>
-      <c r="E11" s="20" t="n">
+      <c r="E11" s="14" t="n">
         <v>31</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -808,10 +857,10 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G11" s="13" t="n">
+      <c r="G11" s="15" t="n">
         <v>37.31</v>
       </c>
-      <c r="O11" s="13">
+      <c r="O11" s="15">
         <f>E11*G11</f>
         <v/>
       </c>
@@ -820,19 +869,24 @@
           <t>https://ibgoetz.sharepoint.com/:b:/s/IBG_Gewerbe/IQC30NCBU9A_TKQDbCNJgepgAZR8CeUhfyKy5Hk9NjtHBN0?e=96lFEy</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="Q11" s="19" t="inlineStr">
         <is>
           <t>https://www.metz-connect.com/home/produkte/p-cabling/anschlussdosen/rj45.ea.de.html</t>
         </is>
       </c>
+      <c r="R11" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Datennetzwerktechnik/Netzwerkkomponente/Kommunikationsanschlussdosen/Kupfer/Metz-Connect-Anschlussdose-Cat-6A-TN-E-DATmod-2Up0::144962.html</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="210" customHeight="1">
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">UP, Daten-Anschlussdose, Cat.6, 2x RJ45, Arbeitsplätze </t>
         </is>
       </c>
-      <c r="E12" s="20" t="n">
+      <c r="E12" s="14" t="n">
         <v>657</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -840,10 +894,10 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G12" s="13" t="n">
+      <c r="G12" s="15" t="n">
         <v>37.31</v>
       </c>
-      <c r="O12" s="13">
+      <c r="O12" s="15">
         <f>E12*G12</f>
         <v/>
       </c>
@@ -852,14 +906,19 @@
           <t>https://ibgoetz.sharepoint.com/:b:/s/IBG_Gewerbe/IQC30NCBU9A_TKQDbCNJgepgAZR8CeUhfyKy5Hk9NjtHBN0?e=96lFEy</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="Q12" s="19" t="inlineStr">
         <is>
           <t>https://www.metz-connect.com/home/produkte/p-cabling/anschlussdosen/rj45.ea.de.html</t>
         </is>
       </c>
+      <c r="R12" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Datennetzwerktechnik/Netzwerkkomponente/Kommunikationsanschlussdosen/Kupfer/Metz-Connect-Anschlussdose-Cat-6A-TN-E-DATmod-2Up0::144962.html</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="45" customHeight="1">
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>Aufputz-Kappe 1fach</t>
         </is>
@@ -872,27 +931,27 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G13" s="13" t="n">
+      <c r="G13" s="15" t="n">
         <v>23.51</v>
       </c>
-      <c r="O13" s="13">
+      <c r="O13" s="15">
         <f>E13*G13</f>
         <v/>
       </c>
       <c r="P13" s="5" t="n"/>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>https://www.jung.de/de/online-katalog/2515061/</t>
+      <c r="Q13" s="19" t="inlineStr">
+        <is>
+          <t>https://www.metz-connect.com/home/produkte/p-cabling/anschlussdosen/rj45.ea.de.html</t>
         </is>
       </c>
     </row>
     <row r="14" ht="225" customHeight="1">
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Abdeckung für IAE/UAE-Anschlussdosen, 2 x 8-polig, mit Schriftfeld, Thermoplast, Serie LS, alpinweiß</t>
         </is>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E14" s="14" t="n">
         <v>982</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -900,10 +959,10 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G14" s="13" t="n">
+      <c r="G14" s="15" t="n">
         <v>13.09</v>
       </c>
-      <c r="O14" s="13">
+      <c r="O14" s="15">
         <f>E14*G14</f>
         <v/>
       </c>
@@ -912,19 +971,19 @@
           <t>https://ibgoetz.sharepoint.com/:b:/s/IBG_Gewerbe/IQA-aqeJ2vRKQI91lZgVitbGAavU4rj4EJLVJxKkA_I0pNI?e=qfSxb5</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>https://www.jung.de/de/online-katalog/2515061/</t>
+      <c r="R14" s="19" t="inlineStr">
+        <is>
+          <t>https://www.gunstigesschaltermaterial.de/jung-ls-969-2-ua-ww.html</t>
         </is>
       </c>
     </row>
     <row r="15" ht="195" customHeight="1">
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>Rahmen 1fach, LS 990, IP 44, Duroplast, alpinweiß, senkrechte und waagerechte Montage</t>
         </is>
       </c>
-      <c r="E15" s="20" t="n">
+      <c r="E15" s="14" t="n">
         <v>982</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -932,17 +991,22 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G15" s="13" t="n">
+      <c r="G15" s="15" t="n">
         <v>6.26</v>
       </c>
-      <c r="O15" s="13">
+      <c r="O15" s="15">
         <f>E15*G15</f>
         <v/>
       </c>
       <c r="P15" s="8" t="n"/>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>https://www.jung.de/de/online-katalog/2515073/</t>
+      <c r="Q15" s="19" t="inlineStr">
+        <is>
+          <t>https://www.jung-group.com/en-DE/p/Frame-1-gang-white/LS-981-WW</t>
+        </is>
+      </c>
+      <c r="R15" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektro-wandelt.de/JUNG-LS981WW-Rahmen-1fach-LS-990-IP-44-Duroplast-alpinweiss-senkrechte-und-waagerechte-Montage.html</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
@@ -950,62 +1014,41 @@
           <t>Gesamt dosen</t>
         </is>
       </c>
-      <c r="Z15" s="14">
+      <c r="Z15" s="17">
         <f>O5+O6+O7+O8+O9+O10+O11+O12+O13+O14+O15</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>Daten-Anschlussdose LWL Duplex-SC, UP</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Stk</t>
-        </is>
-      </c>
-      <c r="G16" s="13" t="n">
-        <v>89.5</v>
-      </c>
-      <c r="O16" s="13">
-        <f>E16*G16</f>
-        <v/>
-      </c>
+      <c r="C16" s="18" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="G16" s="15" t="n"/>
+      <c r="O16" s="15" t="n"/>
       <c r="P16" s="8" t="n"/>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>https://www.metz-connect.com/home/produkte/p-cabling/anschlussdosen/lwl.eb.de.html</t>
-        </is>
-      </c>
     </row>
     <row r="17">
-      <c r="C17" s="6" t="n"/>
+      <c r="C17" s="18" t="n"/>
       <c r="E17" s="11" t="n"/>
-      <c r="G17" s="13" t="n"/>
-      <c r="O17" s="13" t="n"/>
+      <c r="G17" s="15" t="n"/>
+      <c r="O17" s="15" t="n"/>
       <c r="P17" s="8" t="n"/>
     </row>
     <row r="18">
-      <c r="C18" s="6" t="n"/>
+      <c r="C18" s="18" t="n"/>
       <c r="E18" s="11" t="n"/>
-      <c r="G18" s="13" t="n"/>
-      <c r="O18" s="13" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="O18" s="15" t="n"/>
       <c r="P18" s="8" t="n"/>
     </row>
     <row r="19" ht="76.5" customHeight="1">
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">Kabelrinne, Höhe 60 mm, Breite 100 mm 
 </t>
         </is>
       </c>
       <c r="D19" s="2" t="n"/>
-      <c r="E19" s="21" t="n">
+      <c r="E19" s="20" t="n">
         <v>229.94</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1013,7 +1056,7 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G19" s="15" t="n">
+      <c r="G19" s="21" t="n">
         <v>51.2</v>
       </c>
       <c r="H19" s="2" t="n"/>
@@ -1023,25 +1066,30 @@
       <c r="L19" s="2" t="n"/>
       <c r="M19" s="2" t="n"/>
       <c r="N19" s="2" t="n"/>
-      <c r="O19" s="13">
+      <c r="O19" s="15">
         <f>E19*G19</f>
         <v/>
       </c>
       <c r="P19" s="8" t="n"/>
-      <c r="Q19" s="10" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabelrinne-rks-magic-60-ft-3050-100-60-1-ja-zink-stahl-tauchfeuerverzinkt-6047651.html</t>
+      <c r="Q19" s="22" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabelrinne-rks-magic-60-ft-3050-100-60-1-ja-zink-stahl-tauchfeuerverzinkt-6047612.html</t>
+        </is>
+      </c>
+      <c r="R19" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektrotresen.de/Installationsmaterial/Leitungsfuehrung/Kabelrinnen/Rinnen/OBO-Bettermann-Kabelrinne-m-Verbinder-RKSM-610-FS.html</t>
         </is>
       </c>
     </row>
     <row r="20" ht="76.5" customHeight="1">
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">Kabelrinne, Höhe 60 mm, Breite 300 mm </t>
         </is>
       </c>
       <c r="D20" s="2" t="n"/>
-      <c r="E20" s="21" t="n">
+      <c r="E20" s="20" t="n">
         <v>348.89</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1049,7 +1097,7 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G20" s="15" t="n">
+      <c r="G20" s="21" t="n">
         <v>83.75</v>
       </c>
       <c r="H20" s="2" t="n"/>
@@ -1059,19 +1107,19 @@
       <c r="L20" s="2" t="n"/>
       <c r="M20" s="2" t="n"/>
       <c r="N20" s="2" t="n"/>
-      <c r="O20" s="13">
+      <c r="O20" s="15">
         <f>E20*G20</f>
         <v/>
       </c>
       <c r="P20" s="8" t="n"/>
-      <c r="Q20" s="10" t="inlineStr">
+      <c r="Q20" s="22" t="inlineStr">
         <is>
           <t>https://www.obo.de/de-de/produkte/kabelrinne-rks-magic-60-ft-3050-300-60-1-ja-zink-stahl-tauchfeuerverzinkt-6047655.html</t>
         </is>
       </c>
     </row>
     <row r="21" ht="120" customHeight="1">
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">Weitspann-Kabelrinne, Höhe 60 mm, Breite 300 mm </t>
         </is>
@@ -1084,22 +1132,27 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G21" s="15" t="n">
+      <c r="G21" s="21" t="n">
         <v>83.75</v>
       </c>
-      <c r="O21" s="13">
+      <c r="O21" s="15">
         <f>E21*G21</f>
         <v/>
       </c>
       <c r="P21" s="8" t="n"/>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/weitspannkabelrinne-wksg-163-ft-6000-300-160-2-ja-zink-stahl-tauchfeuerverzinkt-6098506.html</t>
+      <c r="Q21" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen/kabelrinnen-weitspann</t>
+        </is>
+      </c>
+      <c r="R21" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektrotools.de/Produkt/6098505-OBO-Bettermann-Weitspannkabelrinne-160x300x6000mm-WKSG-163-FS</t>
         </is>
       </c>
     </row>
     <row r="22" ht="105" customHeight="1">
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="18" t="inlineStr">
         <is>
           <t>Gitterrinne, IBG, Decke, Höhe 55 mm, Breite 200 mm</t>
         </is>
@@ -1112,22 +1165,22 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G22" s="13" t="n">
+      <c r="G22" s="15" t="n">
         <v>28.8</v>
       </c>
-      <c r="O22" s="13">
+      <c r="O22" s="15">
         <f>E22*G22</f>
         <v/>
       </c>
       <c r="P22" s="8" t="n"/>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/gitterrinne-gr-magic-55-ft-3000-200-55-3-9-ja-zink-stahl-tauchfeuerverzinkt-6001420.html</t>
+      <c r="Q22" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektrotresen.de/Installationsmaterial/Leitungsfuehrung/Gitterrinnen/Rinnen/OBO-Bettermann-Gitterkabelrinne-GRM-55-200-FT.html</t>
         </is>
       </c>
     </row>
     <row r="23" ht="105" customHeight="1">
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">Gitterrinne, IBG, Boden, Höhe 55 mm, Breite 200 mm </t>
         </is>
@@ -1140,22 +1193,22 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G23" s="13" t="n">
+      <c r="G23" s="15" t="n">
         <v>28.8</v>
       </c>
-      <c r="O23" s="13">
+      <c r="O23" s="15">
         <f>E23*G23</f>
         <v/>
       </c>
       <c r="P23" s="8" t="n"/>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/gitterrinne-gr-magic-55-ft-3000-200-55-3-9-ja-zink-stahl-tauchfeuerverzinkt-6001420.html</t>
+      <c r="Q23" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektrotresen.de/Installationsmaterial/Leitungsfuehrung/Gitterrinnen/Rinnen/OBO-Bettermann-Gitterkabelrinne-GRM-55-200-FT.html</t>
         </is>
       </c>
     </row>
     <row r="24" ht="105" customHeight="1">
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C24" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">Gitterrinne, IBG, Boden, Höhe 55 mm, Breite 300 mm </t>
         </is>
@@ -1168,43 +1221,43 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G24" s="13" t="n">
-        <v>33.6</v>
-      </c>
-      <c r="O24" s="13">
+      <c r="G24" s="15" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="O24" s="15">
         <f>E24*G24</f>
         <v/>
       </c>
       <c r="P24" s="8" t="n"/>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/gitterrinne-gr-magic-55-ft-3000-300-55-3-9-ja-zink-stahl-tauchfeuerverzinkt-6001424.html</t>
+      <c r="Q24" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Kabel-Leitungen/Kabelzubehoer/Kabeltragsysteme/Gitterrinnen/Gitterrinnen/OBO-Bettermann-Gitterkabelrinne-GRM-55-300-FT::12292.html</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="C25" s="6" t="n"/>
+      <c r="C25" s="18" t="n"/>
       <c r="E25" s="11" t="n"/>
-      <c r="G25" s="13" t="n"/>
-      <c r="O25" s="13" t="n"/>
+      <c r="G25" s="15" t="n"/>
+      <c r="O25" s="15" t="n"/>
       <c r="P25" s="8" t="n"/>
     </row>
     <row r="26">
-      <c r="C26" s="6" t="n"/>
+      <c r="C26" s="18" t="n"/>
       <c r="E26" s="11" t="n"/>
-      <c r="G26" s="13" t="n"/>
-      <c r="O26" s="13" t="n"/>
+      <c r="G26" s="15" t="n"/>
+      <c r="O26" s="15" t="n"/>
       <c r="P26" s="8" t="n"/>
     </row>
     <row r="27">
-      <c r="C27" s="6" t="n"/>
+      <c r="C27" s="18" t="n"/>
       <c r="E27" s="11" t="n"/>
-      <c r="G27" s="13" t="n"/>
-      <c r="O27" s="13" t="n"/>
+      <c r="G27" s="15" t="n"/>
+      <c r="O27" s="15" t="n"/>
       <c r="P27" s="8" t="n"/>
     </row>
     <row r="28" ht="90" customHeight="1">
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C28" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">Datenkabel Kat-7 duplex, 2x4x2xAWG23 </t>
         </is>
@@ -1217,22 +1270,27 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G28" s="13" t="n">
+      <c r="G28" s="15" t="n">
         <v>1.4</v>
       </c>
-      <c r="O28" s="13">
+      <c r="O28" s="15">
         <f>E28*G28</f>
         <v/>
       </c>
       <c r="P28" s="8" t="n"/>
-      <c r="Q28" t="inlineStr">
+      <c r="Q28" s="19" t="inlineStr">
+        <is>
+          <t>https://www.metz-connect.com/home/produkte/p-cabling/kabel-und-leitungen/installationskabel-kupfer.e5.de.html</t>
+        </is>
+      </c>
+      <c r="R28" s="19" t="inlineStr">
         <is>
           <t>https://www.elektro4000.de/Kabel-Leitungen/Kabel/Datenkabel/Metz-Connect-Datenkabel-Kat-7-blau-GC1000-8P-Eca-T500::1068271.html</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="C29" s="16" t="inlineStr">
+      <c r="C29" s="18" t="inlineStr">
         <is>
           <t>Kabelrinne, Höhe 60 mm, Breite 200 mm</t>
         </is>
@@ -1245,21 +1303,24 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G29" s="13" t="n">
-        <v>62.4</v>
-      </c>
-      <c r="O29" s="13">
+      <c r="G29" s="15" t="n"/>
+      <c r="O29" s="15">
         <f>E29*G29</f>
         <v/>
       </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabelrinne-rks-magic-60-ft-3050-200-60-1-ja-zink-stahl-tauchfeuerverzinkt-6047653.html</t>
+      <c r="Q29" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen/kabelrinnen-steckverbindung</t>
+        </is>
+      </c>
+      <c r="R29" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Kabel-Leitungen/Kabelzubehoer/Kabeltragsysteme/Kabelrinnen/Kabelrinnen-Weitspannkabelrinnen/OBO-Bettermann-Kabelrinne-m-Verbinder-RKSM-620-FS::200954.html</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="C30" s="16" t="inlineStr">
+      <c r="C30" s="18" t="inlineStr">
         <is>
           <t>Kabelrinne, Höhe 55 mm, Breite 100 mm</t>
         </is>
@@ -1272,21 +1333,19 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G30" s="13" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="O30" s="13">
+      <c r="G30" s="15" t="n"/>
+      <c r="O30" s="15">
         <f>E30*G30</f>
         <v/>
       </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabelrinne-mks-55-ft-3000-100-1-nein-stahl-tauchfeuerverzinkt-6055410.html</t>
+      <c r="Q30" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen/kabelrinnen-steckverbindung</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="C31" s="16" t="inlineStr">
+      <c r="C31" s="18" t="inlineStr">
         <is>
           <t>Kabelleiter, Höhe 45 mm, Breite 300 mm</t>
         </is>
@@ -1299,21 +1358,24 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G31" s="13" t="n">
-        <v>71.8</v>
-      </c>
-      <c r="O31" s="13">
+      <c r="G31" s="15" t="n"/>
+      <c r="O31" s="15">
         <f>E31*G31</f>
         <v/>
       </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabelleiter-lg-60-3-m-vs-fs-3000-300-1-5-ja-stahl-bandverzinkt-6208541.html</t>
+      <c r="Q31" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelleitern</t>
+        </is>
+      </c>
+      <c r="R31" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Kabel-Leitungen/Kabelzubehoer/Kabeltragsysteme/Kabelleiter/Kabelrinnen-Weitspannkabelleiter/OBO-Bettermann-Kabelleiter-leicht-SL-42-300-FT::28774.html</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="C32" s="16" t="inlineStr">
+      <c r="C32" s="18" t="inlineStr">
         <is>
           <t>Gitterrinne, Höhe 35 mm, Breite 300 mm</t>
         </is>
@@ -1326,21 +1388,24 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G32" s="13" t="n">
-        <v>31.5</v>
-      </c>
-      <c r="O32" s="13">
+      <c r="G32" s="15" t="n"/>
+      <c r="O32" s="15">
         <f>E32*G32</f>
         <v/>
       </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/gitterrinne-gr-35-ft-3000-300-35-3-9-nein-zink-stahl-tauchfeuerverzinkt-6005554.html</t>
+      <c r="Q32" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/gitterrinne-gr-magic-55-ft-3000-100-55-3-9-40-ja-6001416.html</t>
+        </is>
+      </c>
+      <c r="R32" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Kabel-Leitungen/Kabelzubehoer/Kabeltragsysteme/Gitterrinnen/Gitterrinnen/OBO-Bettermann-Gitterrinne-GRM-GRM-35-300-FT::339378.html</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="C33" s="16" t="inlineStr">
+      <c r="C33" s="18" t="inlineStr">
         <is>
           <t>Bogen für Kabelrinne, Höhe 60 mm, Breite 100 mm</t>
         </is>
@@ -1353,21 +1418,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G33" s="13" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="O33" s="13">
+      <c r="G33" s="15" t="n"/>
+      <c r="O33" s="15">
         <f>E33*G33</f>
         <v/>
       </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/bogen-rb-90-610-ft-90-100-60-1-zink-stahl-tauchfeuerverzinkt-7007006.html</t>
+      <c r="Q33" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/produkte/industrieinstallation/kabeltragsysteme/kabelrinnen/formteile-kabelrinnen-steckverbindung/boegen-horizontal-steckverbindung/90-bogen-magic-60-fs.html</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="C34" s="16" t="inlineStr">
+      <c r="C34" s="18" t="inlineStr">
         <is>
           <t>Bogen für Kabelrinne, Höhe 60 mm, Breite 200 mm</t>
         </is>
@@ -1380,21 +1443,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G34" s="13" t="n">
-        <v>47.8</v>
-      </c>
-      <c r="O34" s="13">
+      <c r="G34" s="15" t="n"/>
+      <c r="O34" s="15">
         <f>E34*G34</f>
         <v/>
       </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/bogen-rb-90-620-ft-90-200-60-1-zink-stahl-tauchfeuerverzinkt-7007014.html</t>
+      <c r="Q34" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/produkte/industrieinstallation/kabeltragsysteme/kabelrinnen/formteile-kabelrinnen-steckverbindung/boegen-horizontal-steckverbindung/90-bogen-magic-60-fs.html</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="C35" s="16" t="inlineStr">
+      <c r="C35" s="18" t="inlineStr">
         <is>
           <t>Bogen für Kabelrinne, Höhe 60 mm, Breite 300 mm</t>
         </is>
@@ -1407,21 +1468,24 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G35" s="13" t="n">
-        <v>64.90000000000001</v>
-      </c>
-      <c r="O35" s="13">
+      <c r="G35" s="15" t="n"/>
+      <c r="O35" s="15">
         <f>E35*G35</f>
         <v/>
       </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/bogen-rb-90-630-ft-90-300-60-1-zink-stahl-tauchfeuerverzinkt-7007022.html</t>
+      <c r="Q35" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/produkte/industrieinstallation/kabeltragsysteme/kabelrinnen/formteile-kabelrinnen-steckverbindung/boegen-horizontal-steckverbindung/90-bogen-magic-60-fs.html</t>
+        </is>
+      </c>
+      <c r="R35" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Kabel-Leitungen/Kabeltragsysteme/Kabelrinnen/Boegen/Bogen/OBO-Bettermann-Bogen-90-Grad-RBM-90-630-FS::476892.html</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="C36" s="16" t="inlineStr">
+      <c r="C36" s="18" t="inlineStr">
         <is>
           <t>Bogen für Weitspann-Kabelrinne, Höhe 160 mm, Breite 300 mm</t>
         </is>
@@ -1434,21 +1498,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G36" s="13" t="n">
-        <v>245</v>
-      </c>
-      <c r="O36" s="13">
+      <c r="G36" s="15" t="n"/>
+      <c r="O36" s="15">
         <f>E36*G36</f>
         <v/>
       </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen-zubehoer/bogen</t>
+      <c r="Q36" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen/kabelrinnen-weitspann</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="C37" s="16" t="inlineStr">
+      <c r="C37" s="18" t="inlineStr">
         <is>
           <t>Winkel für Kabelrinne, Höhe 60 mm, Breite 100 mm</t>
         </is>
@@ -1461,21 +1523,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G37" s="13" t="n">
-        <v>34.2</v>
-      </c>
-      <c r="O37" s="13">
+      <c r="G37" s="15" t="n"/>
+      <c r="O37" s="15">
         <f>E37*G37</f>
         <v/>
       </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen-zubehoer/winkel</t>
+      <c r="Q37" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/produkte/industrieinstallation/kabeltragsysteme/kabelrinnen/formteile-kabelrinnen-steckverbindung/boegen-horizontal-steckverbindung/90-bogen-magic-60-fs.html</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="C38" s="16" t="inlineStr">
+      <c r="C38" s="18" t="inlineStr">
         <is>
           <t>Bogen für Kabelleiter, Höhe 45 mm, Breite 300 mm</t>
         </is>
@@ -1488,21 +1548,24 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G38" s="13" t="n">
-        <v>82.5</v>
-      </c>
-      <c r="O38" s="13">
+      <c r="G38" s="15" t="n"/>
+      <c r="O38" s="15">
         <f>E38*G38</f>
         <v/>
       </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelleiter-zubehoer/bogen</t>
+      <c r="Q38" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelleitern</t>
+        </is>
+      </c>
+      <c r="R38" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Kabel-Leitungen/Kabeltragsysteme/Kabelleiter/Boegen/Bogen/OBO-Bettermann-Bogen-90-GRAD-SLB-90-62-300-FT::1259762.html</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="C39" s="16" t="inlineStr">
+      <c r="C39" s="18" t="inlineStr">
         <is>
           <t>Winkel für Kabelleiter, Höhe 45 mm, Breite 300 mm</t>
         </is>
@@ -1515,21 +1578,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G39" s="13" t="n">
-        <v>41</v>
-      </c>
-      <c r="O39" s="13">
+      <c r="G39" s="15" t="n"/>
+      <c r="O39" s="15">
         <f>E39*G39</f>
         <v/>
       </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen-zubehoer/winkel</t>
+      <c r="Q39" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelleitern</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="C40" s="16" t="inlineStr">
+      <c r="C40" s="18" t="inlineStr">
         <is>
           <t>Bogen für Gitterrinne, Höhe 35 mm, Breite 300 mm</t>
         </is>
@@ -1542,21 +1603,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G40" s="13" t="n">
-        <v>29.5</v>
-      </c>
-      <c r="O40" s="13">
+      <c r="G40" s="15" t="n"/>
+      <c r="O40" s="15">
         <f>E40*G40</f>
         <v/>
       </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/gitterrinnen-zubehoer/bogen</t>
+      <c r="Q40" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/produkte/industrieinstallation/kabeltragsysteme/gitterrinnen/zubehoer-gitterrinnen/</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="C41" s="16" t="inlineStr">
+      <c r="C41" s="18" t="inlineStr">
         <is>
           <t>Bogen für Gitterrinne, Höhe 55 mm, Breite 200 mm</t>
         </is>
@@ -1569,21 +1628,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G41" s="13" t="n">
-        <v>32.8</v>
-      </c>
-      <c r="O41" s="13">
+      <c r="G41" s="15" t="n"/>
+      <c r="O41" s="15">
         <f>E41*G41</f>
         <v/>
       </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/gitterrinnen-zubehoer/bogen</t>
+      <c r="Q41" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/produkte/industrieinstallation/kabeltragsysteme/gitterrinnen/zubehoer-gitterrinnen/</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="C42" s="16" t="inlineStr">
+      <c r="C42" s="18" t="inlineStr">
         <is>
           <t>Bogen für Kabelrinne, Höhe 55 mm, Breite 100 mm</t>
         </is>
@@ -1596,21 +1653,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G42" s="13" t="n">
-        <v>30.4</v>
-      </c>
-      <c r="O42" s="13">
+      <c r="G42" s="15" t="n"/>
+      <c r="O42" s="15">
         <f>E42*G42</f>
         <v/>
       </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/bogen-rb-90-610-ft-90-100-60-1-zink-stahl-tauchfeuerverzinkt-7007006.html</t>
+      <c r="Q42" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/produkte/industrieinstallation/kabeltragsysteme/kabelrinnen/formteile-kabelrinnen-steckverbindung/boegen-horizontal-steckverbindung/90-bogen-magic-60-fs.html</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="C43" s="16" t="inlineStr">
+      <c r="C43" s="18" t="inlineStr">
         <is>
           <t>Anschluss Kabelrinne 60/100 &gt; Abgang 100 mm</t>
         </is>
@@ -1623,21 +1678,24 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G43" s="13" t="n">
-        <v>25.8</v>
-      </c>
-      <c r="O43" s="13">
+      <c r="G43" s="15" t="n"/>
+      <c r="O43" s="15">
         <f>E43*G43</f>
         <v/>
       </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen-zubehoer/anschluss</t>
+      <c r="Q43" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen/kabelrinnen-steckverbindung</t>
+        </is>
+      </c>
+      <c r="R43" s="19" t="inlineStr">
+        <is>
+          <t>https://www.tandmore.de/Installation/OBO-Bettermann/Sonstiges/OBO-Bettermann-6042111-RAA-610-FS-f-Kabelrinne-60x100-Anbau-Abzweigstueck::1027860.html</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="C44" s="16" t="inlineStr">
+      <c r="C44" s="18" t="inlineStr">
         <is>
           <t>Anschluss Kabelrinne 60/300 &gt; Abgang 300 mm</t>
         </is>
@@ -1650,21 +1708,24 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G44" s="13" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="O44" s="13">
+      <c r="G44" s="15" t="n"/>
+      <c r="O44" s="15">
         <f>E44*G44</f>
         <v/>
       </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen-zubehoer/anschluss</t>
+      <c r="Q44" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen/kabelrinnen-steckverbindung</t>
+        </is>
+      </c>
+      <c r="R44" s="19" t="inlineStr">
+        <is>
+          <t>https://www.tandmore.de/Installation/OBO-Bettermann/Sonstiges/OBO-Bettermann-6042111-RAA-610-FS-f-Kabelrinne-60x100-Anbau-Abzweigstueck::1027860.html</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="C45" s="16" t="inlineStr">
+      <c r="C45" s="18" t="inlineStr">
         <is>
           <t>Anschluss Kabelrinne 55/100 &gt; Abgang 100 mm</t>
         </is>
@@ -1677,21 +1738,24 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G45" s="13" t="n">
-        <v>25.8</v>
-      </c>
-      <c r="O45" s="13">
+      <c r="G45" s="15" t="n"/>
+      <c r="O45" s="15">
         <f>E45*G45</f>
         <v/>
       </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen-zubehoer/anschluss</t>
+      <c r="Q45" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen/kabelrinnen-steckverbindung</t>
+        </is>
+      </c>
+      <c r="R45" s="19" t="inlineStr">
+        <is>
+          <t>https://www.tandmore.de/Installation/OBO-Bettermann/Sonstiges/OBO-Bettermann-6042111-RAA-610-FS-f-Kabelrinne-60x100-Anbau-Abzweigstueck::1027860.html</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="C46" s="16" t="inlineStr">
+      <c r="C46" s="18" t="inlineStr">
         <is>
           <t>T-Abgang Kabelrinne 60/100 &gt; Abgang 100 mm</t>
         </is>
@@ -1704,21 +1768,24 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G46" s="13" t="n">
-        <v>46.2</v>
-      </c>
-      <c r="O46" s="13">
+      <c r="G46" s="15" t="n"/>
+      <c r="O46" s="15">
         <f>E46*G46</f>
         <v/>
       </c>
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen-zubehoer/t-stueck</t>
+      <c r="Q46" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen/kabelrinnen-steckverbindung</t>
+        </is>
+      </c>
+      <c r="R46" s="19" t="inlineStr">
+        <is>
+          <t>https://www.alles-mit-stecker.de/Installationsmaterial/Kabeltragsysteme/T-Stueck-fuer-Kabelrinne/OBO-Bettermann-T-Abzweigstueck-60x300mm-RTM-630-FS::273169.html</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="C47" s="16" t="inlineStr">
+      <c r="C47" s="18" t="inlineStr">
         <is>
           <t>T-Abgang Kabelleiter 45/300 &gt; Abgang 300 mm</t>
         </is>
@@ -1731,21 +1798,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G47" s="13" t="n">
-        <v>118</v>
-      </c>
-      <c r="O47" s="13">
+      <c r="G47" s="15" t="n"/>
+      <c r="O47" s="15">
         <f>E47*G47</f>
         <v/>
       </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen-zubehoer/t-stueck</t>
+      <c r="Q47" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelleitern</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="C48" s="16" t="inlineStr">
+      <c r="C48" s="18" t="inlineStr">
         <is>
           <t>Winkel oben/unten Kabelrinne 60/100, normal</t>
         </is>
@@ -1758,21 +1823,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G48" s="13" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="O48" s="13">
+      <c r="G48" s="15" t="n"/>
+      <c r="O48" s="15">
         <f>E48*G48</f>
         <v/>
       </c>
-      <c r="Q48" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen-zubehoer/winkel</t>
+      <c r="Q48" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/produkte/industrieinstallation/kabeltragsysteme/kabelrinnen/formteile-kabelrinnen-steckverbindung/boegen-horizontal-steckverbindung/90-bogen-magic-60-fs.html</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="C49" s="16" t="inlineStr">
+      <c r="C49" s="18" t="inlineStr">
         <is>
           <t>Winkel oben/unten Kabelrinne 60/300, normal</t>
         </is>
@@ -1785,21 +1848,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G49" s="13" t="n">
-        <v>56.4</v>
-      </c>
-      <c r="O49" s="13">
+      <c r="G49" s="15" t="n"/>
+      <c r="O49" s="15">
         <f>E49*G49</f>
         <v/>
       </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/kabelrinnen-zubehoer/winkel</t>
+      <c r="Q49" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/produkte/industrieinstallation/kabeltragsysteme/kabelrinnen/formteile-kabelrinnen-steckverbindung/boegen-horizontal-steckverbindung/90-bogen-magic-60-fs.html</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="C50" s="16" t="inlineStr">
+      <c r="C50" s="18" t="inlineStr">
         <is>
           <t>T-Hängestiel B = 400 mm</t>
         </is>
@@ -1812,21 +1873,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G50" s="13" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="O50" s="13">
+      <c r="G50" s="15" t="n"/>
+      <c r="O50" s="15">
         <f>E50*G50</f>
         <v/>
       </c>
-      <c r="Q50" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/wand-und-stielausleger-aw-15-ft-110-1-5-zink-6420656.html</t>
+      <c r="Q50" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/tragkonstruktionen/abhaengungen-und-buegel/halter-und-befestigungen</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="C51" s="16" t="inlineStr">
+      <c r="C51" s="18" t="inlineStr">
         <is>
           <t>Kabelbahnhalter, Wandmontage, L-Form, W=200 mm</t>
         </is>
@@ -1839,21 +1898,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G51" s="13" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="O51" s="13">
+      <c r="G51" s="15" t="n"/>
+      <c r="O51" s="15">
         <f>E51*G51</f>
         <v/>
       </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/tragkonstruktionen</t>
+      <c r="Q51" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/tragkonstruktionen/abhaengungen-und-buegel/halter-und-befestigungen</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="C52" s="16" t="inlineStr">
+      <c r="C52" s="18" t="inlineStr">
         <is>
           <t>Kabelbahnhalter mit 1 Hängestiel, W=100 mm</t>
         </is>
@@ -1866,21 +1923,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G52" s="13" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="O52" s="13">
+      <c r="G52" s="15" t="n"/>
+      <c r="O52" s="15">
         <f>E52*G52</f>
         <v/>
       </c>
-      <c r="Q52" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/tragkonstruktionen</t>
+      <c r="Q52" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/tragkonstruktionen/abhaengungen-und-buegel/halter-und-befestigungen</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="C53" s="16" t="inlineStr">
+      <c r="C53" s="18" t="inlineStr">
         <is>
           <t>Kabelbahnhalter mit 1 Hängestiel, W=200 mm</t>
         </is>
@@ -1893,21 +1948,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G53" s="13" t="n">
-        <v>11.9</v>
-      </c>
-      <c r="O53" s="13">
+      <c r="G53" s="15" t="n"/>
+      <c r="O53" s="15">
         <f>E53*G53</f>
         <v/>
       </c>
-      <c r="Q53" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/tragkonstruktionen</t>
+      <c r="Q53" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/tragkonstruktionen/abhaengungen-und-buegel/halter-und-befestigungen</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="C54" s="16" t="inlineStr">
+      <c r="C54" s="18" t="inlineStr">
         <is>
           <t>Kabelbahnhalter mit 1 Hängestiel, W=300 mm</t>
         </is>
@@ -1920,21 +1973,19 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G54" s="13" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="O54" s="13">
+      <c r="G54" s="15" t="n"/>
+      <c r="O54" s="15">
         <f>E54*G54</f>
         <v/>
       </c>
-      <c r="Q54" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/tragkonstruktionen</t>
+      <c r="Q54" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/kabeltragsysteme/tragkonstruktionen/abhaengungen-und-buegel/halter-und-befestigungen</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="C55" s="16" t="inlineStr">
+      <c r="C55" s="18" t="inlineStr">
         <is>
           <t>Brüstungskanal, bauseits, 50 Hertz</t>
         </is>
@@ -1947,21 +1998,19 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G55" s="13" t="n">
-        <v>19.5</v>
-      </c>
-      <c r="O55" s="13">
+      <c r="G55" s="15" t="n"/>
+      <c r="O55" s="15">
         <f>E55*G55</f>
         <v/>
       </c>
-      <c r="Q55" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/installation-und-gebaeudesysteme/bruestungskanalsysteme</t>
+      <c r="Q55" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/geraeteeinbaukanaele-und-saeulen/geraeteeinbaukanaele/geraeteeinbaukanaele-rapid-80</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="C56" s="16" t="inlineStr">
+      <c r="C56" s="18" t="inlineStr">
         <is>
           <t>Sammelhalter, 2 Stk/m, 80 mm x 170 mm</t>
         </is>
@@ -1974,21 +2023,19 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G56" s="13" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="O56" s="13">
+      <c r="G56" s="15" t="n"/>
+      <c r="O56" s="15">
         <f>E56*G56</f>
         <v/>
       </c>
-      <c r="Q56" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/sammelhalter-2-stueck-m-pfsh-80-170</t>
+      <c r="Q56" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/de-de/produkte/geraeteeinbaukanaele-und-saeulen/geraeteeinbaukanaele/geraeteeinbaukanaele-rapid-80</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="C57" s="16" t="inlineStr">
+      <c r="C57" s="18" t="inlineStr">
         <is>
           <t>Brüstungskanal Rapid 80, Höhe 70 x Breite 110 mm</t>
         </is>
@@ -2001,23 +2048,21 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G57" s="13" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="O57" s="13">
+      <c r="G57" s="15" t="n"/>
+      <c r="O57" s="15">
         <f>E57*G57</f>
         <v/>
       </c>
-      <c r="Q57" t="inlineStr">
+      <c r="Q57" s="19" t="inlineStr">
         <is>
           <t>https://www.obo.de/de-de/produkte/geraeteeinbaukanal-rapid-80-kanalbreite-110-kanalhoehe-70-2000-reinweiss-ral-9010-6274300.html</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="C58" s="16" t="inlineStr">
-        <is>
-          <t>Fußbodenkanaldose UDHOME, mit Blinddeckel, rund</t>
+      <c r="C58" s="18" t="inlineStr">
+        <is>
+          <t>Fußbodenkanaldose UDHOME2, mit Blinddeckel, rund</t>
         </is>
       </c>
       <c r="E58" s="11" t="n">
@@ -2028,21 +2073,24 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G58" s="13" t="n">
-        <v>186</v>
-      </c>
-      <c r="O58" s="13">
+      <c r="G58" s="15" t="n"/>
+      <c r="O58" s="15">
         <f>E58*G58</f>
         <v/>
       </c>
-      <c r="Q58" t="inlineStr">
-        <is>
-          <t>https://www.obo.de/de-de/produkte/bodensteckdose-udhome2-vt2-7427097.html</t>
+      <c r="Q58" s="19" t="inlineStr">
+        <is>
+          <t>https://www.obo.de/produkte/gebaeudeinstallation/produkthighlights/udhome-bodentanks-und-bodensteckdosen/udhome2-bodensteckdose/</t>
+        </is>
+      </c>
+      <c r="R58" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Installationsmaterial/Unterflursysteme/Geraeteeinsaetze/OBO-Bettermann-Bodensteckdose-UDHOME2-VT2::1584327.html</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="C59" s="16" t="inlineStr">
+      <c r="C59" s="18" t="inlineStr">
         <is>
           <t>SAA Datenkabel Kat-7 duplex, 2x4x2xAWG23</t>
         </is>
@@ -2055,21 +2103,24 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G59" s="13" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="O59" s="13">
+      <c r="G59" s="15" t="n"/>
+      <c r="O59" s="15">
         <f>E59*G59</f>
         <v/>
       </c>
-      <c r="Q59" t="inlineStr">
+      <c r="Q59" s="19" t="inlineStr">
         <is>
           <t>https://www.metz-connect.com/home/produkte/p-cabling/kabel-und-leitungen/installationskabel-kupfer.e5.de.html</t>
         </is>
       </c>
+      <c r="R59" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektro4000.de/Kabel-Leitungen/Kabel/Datenkabel/Metz-Connect-Datenkabel-Kat-7-blau-GC1000-8P-Eca-T500::1068271.html</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="C60" s="16" t="inlineStr">
+      <c r="C60" s="18" t="inlineStr">
         <is>
           <t>Leitung Lautsprecher J-Y(St)Y 4x2x0,8</t>
         </is>
@@ -2082,21 +2133,19 @@
           <t>m</t>
         </is>
       </c>
-      <c r="G60" s="13" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="O60" s="13">
+      <c r="G60" s="15" t="n"/>
+      <c r="O60" s="15">
         <f>E60*G60</f>
         <v/>
       </c>
-      <c r="Q60" t="inlineStr">
-        <is>
-          <t>https://www.metz-connect.com/home/produkte/p-cabling/kabel-und-leitungen.e1.de.html</t>
+      <c r="R60" s="19" t="inlineStr">
+        <is>
+          <t>https://www.elektroversand-schmidt.de/Kabel-Leitungen/Fernmeldeleitung/Fernmeldekabel-0-8mm/Fernmeldekabel-J-Y-St-Y-4x2x0-8-500m-Trommel.html</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="C61" s="16" t="inlineStr">
+      <c r="C61" s="18" t="inlineStr">
         <is>
           <t>Netzwerkschrank IBG 42 HE (Rittal VX IT, 800x1000)</t>
         </is>
@@ -2109,48 +2158,58 @@
           <t>Stk</t>
         </is>
       </c>
-      <c r="G61" s="13" t="n">
-        <v>1335</v>
-      </c>
-      <c r="O61" s="13">
+      <c r="G61" s="15" t="n"/>
+      <c r="O61" s="15">
         <f>E61*G61</f>
         <v/>
       </c>
-      <c r="Q61" t="inlineStr">
-        <is>
-          <t>https://www.rittal.com/de-de/products/PG0001SCHRANKSYSTEME1/PG0758VX_ITSCHRANKSYSTEME</t>
+      <c r="Q61" s="19" t="inlineStr">
+        <is>
+          <t>https://www.rittal.com/de-de/products/PG20231215ITI101/PG20240402ITI203/PRO106268</t>
+        </is>
+      </c>
+      <c r="R61" s="19" t="inlineStr">
+        <is>
+          <t>https://www.serverschrank.de/19-Serverschrank-VX-IT-von-RITTAL-42-HE-800x1000-mm-perforierte-Tueren-oSeitenwaende-lichtgrau</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="C63" s="17" t="inlineStr">
+      <c r="C63" s="23" t="inlineStr">
         <is>
           <t>GESAMTSUMME (netto)</t>
         </is>
       </c>
-      <c r="O63" s="18">
+      <c r="O63" s="24">
         <f>SUM(O5:O61)</f>
         <v/>
       </c>
     </row>
-    <row r="64">
-      <c r="Y64" s="19" t="inlineStr">
-        <is>
-          <t>Hinweis:</t>
-        </is>
-      </c>
-    </row>
     <row r="65">
-      <c r="Y65" s="16" t="inlineStr">
-        <is>
-          <t>Preise sind unverbindliche Listenrichtpreise (netto, ohne Skonto/Projektrabatt).</t>
+      <c r="C65" s="25" t="inlineStr">
+        <is>
+          <t>Hinweise:</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="Y66" s="16" t="inlineStr">
-        <is>
-          <t>Produkte beispielhaft aus dem Hersteller-Sortiment ausgewählt — finale Auswahl vor Bestellung verifizieren.</t>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Spalte G (EP) bewusst leer — Preise bitte direkt von der verlinkten Seite (Spalte R bzw. Q) eintragen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Q = Hersteller-Produktseite, R = Händler-Shop mit Preis. Alle Links auf Existenz geprüft (indexiert).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Einige OBO-Kleinteile verlinken auf die Produkt-/Kategorieseite der jeweiligen Serie — dort exakte Variante wählen.</t>
         </is>
       </c>
     </row>
@@ -2158,65 +2217,84 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" display="https://ibgoetz.sharepoint.com/:b:/s/IBG_Gewerbe/IQC30NCBU9A_TKQDbCNJgepgAZR8CeUhfyKy5Hk9NjtHBN0?e=96lFEy" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" display="https://ibgoetz.sharepoint.com/:b:/s/IBG_Gewerbe/IQC30NCBU9A_TKQDbCNJgepgAZR8CeUhfyKy5Hk9NjtHBN0?e=96lFEy" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" display="https://ibgoetz.sharepoint.com/:b:/s/IBG_Gewerbe/IQC30NCBU9A_TKQDbCNJgepgAZR8CeUhfyKy5Hk9NjtHBN0?e=96lFEy" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" display="https://ibgoetz.sharepoint.com/:b:/s/IBG_Gewerbe/IQC30NCBU9A_TKQDbCNJgepgAZR8CeUhfyKy5Hk9NjtHBN0?e=96lFEy" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R58" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R59" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R60" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R61" r:id="rId80"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>